<commit_message>
xlsx files nicer formatting
</commit_message>
<xml_diff>
--- a/technical-triz/innovation-checklist/assets/TRU_ISQ_DE.xlsx
+++ b/technical-triz/innovation-checklist/assets/TRU_ISQ_DE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jens\dev\github\truinorva\triz-skills\technical-triz\innovation-checklist\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075B004F-E2EF-4EFC-B991-2F0CD1CC6750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C14A38-AF8E-4E54-9448-4F49E951D200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,7 +125,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,13 +141,39 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -177,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -186,6 +212,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -528,16 +560,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="3"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="5"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">

</xml_diff>